<commit_message>
Update sensor defaults and regenerate wiki estimates
</commit_message>
<xml_diff>
--- a/alpha calculations.xlsx
+++ b/alpha calculations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jpl365prod-my.sharepoint.com/personal/mark_a_lindeman_jpl_nasa_gov/Documents/Documents/neutrino/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{2CE06A65-07B9-4854-9676-C2C0D0A39068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B65B524-A11C-42D8-AE9D-D6E9B3918D80}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="8_{2CE06A65-07B9-4854-9676-C2C0D0A39068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0768F95-5429-4A7C-BD86-C52001D3210A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1F8C9631-E3A8-4EDD-9FFD-210F3E74B3BA}"/>
+    <workbookView minimized="1" xWindow="1296" yWindow="1404" windowWidth="14376" windowHeight="9792" xr2:uid="{1F8C9631-E3A8-4EDD-9FFD-210F3E74B3BA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t>NEP</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t>not given in aper</t>
+  </si>
+  <si>
+    <t>T= 200</t>
   </si>
 </sst>
 </file>
@@ -678,6 +681,11 @@
         <v>21</v>
       </c>
     </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+    </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>26</v>
@@ -739,7 +747,7 @@
       <c r="A18" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="1">
+      <c r="C18" s="1">
         <v>20000</v>
       </c>
       <c r="D18" t="s">

</xml_diff>